<commit_message>
fix(ba-kit): sửa số thứ tự cột # trong sheet Sample của file mẫu
Cột # rows 9-19 đang là 1,2,3,4,3,4,5,6,3,4,4 với kiểu dữ liệu lẫn lộn
int/string. Lỗi có sẵn trong template gốc của công ty — cả Sample lẫn
Login_Sample đều mang cùng dãy số này, nhiều khả năng do sao chép từ một màn
wizard có đánh số lại theo từng step.

Đổi thành 1..11 dạng số nguyên. Sheet sinh ra từ populate không bị ảnh hưởng vì
cột H được ghi đè, nhưng người điền tay sẽ thấy template đúng.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ba-kit/requirement-to-flow/sample/sample_basic_design.xlsx
+++ b/ba-kit/requirement-to-flow/sample/sample_basic_design.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -165,8 +165,19 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1F5C1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -230,6 +241,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDAEEF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -885,7 +901,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1207,6 +1223,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="12" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="12" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="12" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -15543,10 +15574,8 @@
       <c r="E10" s="31" t="n"/>
       <c r="F10" s="31" t="n"/>
       <c r="G10" s="31" t="n"/>
-      <c r="H10" s="36" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="H10" s="36" t="n">
+        <v>2</v>
       </c>
       <c r="I10" s="37" t="n"/>
       <c r="J10" s="37" t="n"/>
@@ -15656,10 +15685,8 @@
       <c r="E13" s="31" t="n"/>
       <c r="F13" s="31" t="n"/>
       <c r="G13" s="31" t="n"/>
-      <c r="H13" s="36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="H13" s="36" t="n">
+        <v>5</v>
       </c>
       <c r="I13" s="37" t="n"/>
       <c r="J13" s="37" t="n"/>
@@ -15695,10 +15722,8 @@
       <c r="E14" s="31" t="n"/>
       <c r="F14" s="31" t="n"/>
       <c r="G14" s="31" t="n"/>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="H14" s="36" t="n">
+        <v>6</v>
       </c>
       <c r="I14" s="37" t="n"/>
       <c r="J14" s="37" t="n"/>
@@ -15735,7 +15760,7 @@
       <c r="F15" s="31" t="n"/>
       <c r="G15" s="31" t="n"/>
       <c r="H15" s="36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I15" s="37" t="n"/>
       <c r="J15" s="37" t="n"/>
@@ -15772,7 +15797,7 @@
       <c r="F16" s="31" t="n"/>
       <c r="G16" s="31" t="n"/>
       <c r="H16" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I16" s="37" t="n"/>
       <c r="J16" s="37" t="n"/>
@@ -15808,10 +15833,8 @@
       <c r="E17" s="31" t="n"/>
       <c r="F17" s="31" t="n"/>
       <c r="G17" s="31" t="n"/>
-      <c r="H17" s="36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="H17" s="36" t="n">
+        <v>9</v>
       </c>
       <c r="I17" s="37" t="n"/>
       <c r="J17" s="37" t="n"/>
@@ -15847,10 +15870,8 @@
       <c r="E18" s="31" t="n"/>
       <c r="F18" s="31" t="n"/>
       <c r="G18" s="31" t="n"/>
-      <c r="H18" s="36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="H18" s="36" t="n">
+        <v>10</v>
       </c>
       <c r="I18" s="37" t="n"/>
       <c r="J18" s="37" t="n"/>
@@ -15887,7 +15908,7 @@
       <c r="F19" s="31" t="n"/>
       <c r="G19" s="31" t="n"/>
       <c r="H19" s="36" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I19" s="41" t="n"/>
       <c r="J19" s="41" t="n"/>
@@ -26512,23 +26533,71 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="64" t="n"/>
-      <c r="B10" s="67" t="n"/>
-      <c r="C10" s="65" t="n"/>
-      <c r="D10" s="65" t="n"/>
-      <c r="E10" s="65" t="n"/>
-      <c r="F10" s="65" t="n"/>
-      <c r="G10" s="65" t="n"/>
-      <c r="H10" s="65" t="n"/>
-      <c r="I10" s="65" t="n"/>
-      <c r="J10" s="65" t="n"/>
-      <c r="K10" s="75" t="n"/>
-      <c r="L10" s="75" t="n"/>
-      <c r="M10" s="65" t="n"/>
-      <c r="N10" s="65" t="n"/>
-      <c r="O10" s="67" t="n"/>
-      <c r="P10" s="65" t="n"/>
+    <row r="10" ht="30" customHeight="1" s="84">
+      <c r="A10" s="128" t="inlineStr">
+        <is>
+          <t>CHG-0005</t>
+        </is>
+      </c>
+      <c r="B10" s="129" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C10" s="130" t="inlineStr">
+        <is>
+          <t>BA Agent</t>
+        </is>
+      </c>
+      <c r="D10" s="130" t="inlineStr">
+        <is>
+          <t>MASTER_STANDARDIZATION</t>
+        </is>
+      </c>
+      <c r="E10" s="130" t="inlineStr"/>
+      <c r="F10" s="130" t="inlineStr"/>
+      <c r="G10" s="130" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="H10" s="130" t="inlineStr">
+        <is>
+          <t>Cot # rows 9-19</t>
+        </is>
+      </c>
+      <c r="I10" s="130" t="inlineStr">
+        <is>
+          <t>Danh lai so thu tu 1..11 (truoc do la 1,2,3,4,3,4,5,6,3,4,4 - loi co san trong template goc)</t>
+        </is>
+      </c>
+      <c r="J10" s="130" t="inlineStr">
+        <is>
+          <t>Feedback user 23/09/2026</t>
+        </is>
+      </c>
+      <c r="K10" s="131" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="L10" s="131" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="M10" s="130" t="inlineStr">
+        <is>
+          <t>WAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="N10" s="130" t="inlineStr"/>
+      <c r="O10" s="132" t="inlineStr"/>
+      <c r="P10" s="130" t="inlineStr">
+        <is>
+          <t>Loi co san o ca Sample lan Login_Sample cua ban goc, khong phai do thay doi truoc do</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="64" t="n"/>

</xml_diff>